<commit_message>
docs: update same Excel file — interviewee sign-in → complete evaluation (Login→Evaluate→Submit, queue/lock, 4-criteria rubric 94%, 3-role flow) — same file
</commit_message>
<xml_diff>
--- a/Veridex_Comparison_Merge_Plan.xlsx
+++ b/Veridex_Comparison_Merge_Plan.xlsx
@@ -16,8 +16,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparison'!$A$3:$F$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Comparison'!$1:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merge Checklist'!$A$2:$F$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Website Flow'!$A$2:$E$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merge Checklist'!$A$2:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Website Flow'!$A$2:$E$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,19 +94,13 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <name val="Urbanist"/>
       <b val="1"/>
       <color rgb="0008307F"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -149,12 +143,6 @@
         <bgColor rgb="00FFF1F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -182,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -223,13 +211,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -247,10 +235,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -632,14 +617,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VERIDEX — CODEBASE COMPARISON &amp; MERGE PLAN  (Veridex = Source of Truth)  —  CONSOLIDATED v2 (Home-First + Full Figma UI)</t>
+          <t>VERIDEX — CODEBASE COMPARISON &amp; MERGE PLAN  (Veridex = Source of Truth)  —  CONSOLIDATED + Interviewee Evaluation Complete</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Vercel: github.com/Abdurrahman99max/Veridex  •  Figma: github.com/Abdurrahman99max/Veridexapp  •  Target: Desktop/Veridex System  •  Updated: 2026-09-17 15:00  •  Live: veridex-five.vercel.app &amp; veridexapp.figma.site  •  Commits: c158e63→33dfdc0→63155de→3b9e97e→cde6f34</t>
+          <t>Vercel: github.com/Abdurrahman99max/Veridex  •  Figma: github.com/Abdurrahman99max/Veridexapp  •  Desktop/Veridex System  •  2026-09-17 16:10  •  Live: veridex-five.vercel.app (index-CIfYX0us.js) &amp; veridexapp.figma.site  •  Commits: 33dfdc0→63155de→3b9e97e→cde6f34→6427990→7b5cf03</t>
         </is>
       </c>
     </row>
@@ -676,7 +661,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>STACK</t>
@@ -699,7 +684,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>KEEP Veridex stack (identical)</t>
+          <t>KEEP Veridex stack</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -708,7 +693,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>STACK</t>
@@ -716,7 +701,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Dependencies (unique)</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -726,12 +711,12 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>MUI (@mui/material, @emotion/react, @mui/icons-material), react-router 7.13, react-dnd 16, react-responsive-masonry, react-slick, date-fns — NO Supabase/hono/resend</t>
+          <t>MUI (@mui/material, @emotion/react, @mui/icons-material), react-router 7.13, react-dnd 16, masonry, slick, date-fns — NO Supabase/hono</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>KEEP Veridex deps; drop MUI/masonry/slick (bloated)</t>
+          <t>KEEP Veridex deps; drop MUI/masonry/slick</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
@@ -740,7 +725,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>STACK</t>
@@ -753,7 +738,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>App.tsx View state (landing|gate|application|admin|success|duplicate|seeder|design-system), ?dex/?seed/?design hash — HOME ALWAYS FIRST (landing default, draft banner opt-in)</t>
+          <t>App.tsx View (landing|sign-in|sign-up|candidate|evaluation|admin|design-system), ?dex/?seed/?design — HOME ALWAYS FIRST useState='landing'+ hasDraft banner opt-in</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -763,16 +748,16 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>KEEP View router + home-first guard (useState='landing') + ?design route</t>
+          <t>KEEP View router + home-first + ?design</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>High — fixed in cde6f34</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
+          <t>High — cde6f34</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
@@ -785,7 +770,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>5 commits: c158e63 →33dfdc0 →63155de merge figma-system →3b9e97e mundane ping →cde6f34 home-first+Risk/FinalCTA+WEBSITE_FLOW</t>
+          <t>7b5cf03 HEAD: ...→cde6f34 home-first+Risk/FinalCTA→6427990 EvaluationPanel→7b5cf03 deploy trigger</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -795,7 +780,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Veridex truth preserved; all merges on main, Vercel auto-deploy</t>
+          <t>Veridex truth preserved; Vercel auto-deploy</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -804,7 +789,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
@@ -817,12 +802,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>src/components/{application,landing(10 sections),layout,ui,figma,design-system}, src/database, src/supabase/functions, src/styles (theme/fonts), src/imports/figma, guidelines-figma</t>
+          <t>src/components/{landing(10),auth,dashboard/evaluation,admin,design-system,ui,figma}, src/database, src/supabase/functions, src/styles theme/fonts, imports/figma</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>src/app/components/{design-system,ui,figma}, src/imports/*.svg, src/styles/{fonts,theme,tailwind}</t>
+          <t>src/app/components/{design-system,ui,figma}, src/imports/*.svg, src/styles/{fonts,theme}</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -836,7 +821,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
@@ -849,7 +834,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>vite.config.ts, index.html, .npmrc, .gitignore, vercel.json at root (fixed from src/vercel.json), design-tokens.json</t>
+          <t>vite.config.ts, index.html, .npmrc, vercel.json at root (fixed from src/vercel.json), design-tokens.json</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -868,7 +853,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="44" customHeight="1">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>PAGES / VIEWS</t>
@@ -876,22 +861,22 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>HOME — Landing (consolidated 10 sections)</t>
+          <t>HOME — Landing (10 sections)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>NOW 10 sections in order as Figma: Hero → Reliability → Risk → WhoIsThisFor → HowItWorks → Cohort → WhatWeLookFor → Employer → FinalCTA → Footer (all CTAs wired, no dead href=#)</t>
+          <t>10 sections in Figma order: Hero → Reliability (Alex 8/3/2 94% 96/92/94) → Risk (CVs 3) → WhoIs → How → Cohort 38/50 → What → Employer 3+3 → FinalCTA → Footer (all CTAs wired)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Figma had 9 figma-site sections: verification, Alex card 8/3/2, 94% bars, CVs risk, Who qualifies, How verified, Cohort 38/50, Hire talent, Your profile waiting</t>
+          <t>Figma 9 sections: verification, Alex 8/3/2, 94% bars, CVs risk, Who qualifies, Which track 38/50, Hire talent, Your profile waiting</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>FULL MERGE — every Figma UI present on home, plus Veridex vetting copy</t>
+          <t>FULL MERGE — every Figma UI on home</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -900,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>PAGES / VIEWS</t>
@@ -908,12 +893,12 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Home-first guarantee</t>
+          <t>Home-first</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>App.tsx:23 useState('landing') always; hasDraft banner 'Resume application →' opt-in; useEffect only switches on ?dex/?seed/?design</t>
+          <t>App.tsx:23 useState='landing' always; hasDraft sticky Resume banner opt-in; useEffect only switches on ?dex/?seed/?design</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -923,16 +908,16 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>ENFORCED: home loads before any gate/application</t>
+          <t>ENFORCED: home before any gate</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>High — user req</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PAGES / VIEWS</t>
@@ -940,635 +925,635 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Application Flow</t>
+          <t>Auth — sign in/up</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>EntryGate (Not for Everyone) → Step1Eligibility → Step2SkillProof (12 domains, acceptable/rejection, 20w rationale, proofUrl) → Step3Verification/Commitment → ReviewStep → Success/Duplicate → localStorage vdx_draft</t>
+          <t>/auth/sign-up (fullName|email|university|gradYear VxSelect|skillCategory 12 domains acceptable/rejection|proofUrl|rationale≥20w|track Core|Prep) → POST /submit-application VX-C|P APPLIED → /auth/sign-in; /auth/sign-in email+OTP → role redirect</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>NEW Figma VxInput forms → redirect</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>High — core req</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>PAGES / VIEWS</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Dashboards 3 roles</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>/dashboard/candidate (read-only VxAvatar verified, 94% bars, APPLIED pill) | /dashboard/evaluation (queue + EvaluationPanel) | /dashboard/admin (AdminHub lite) | /?design catalogue 1475 lines</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>None / catalogue only</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>3 views candidate|evaluation|admin distinct</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>COMPONENTS</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>UI library</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Radix + shadcn ui/* 45 files, utils.ts, use-mobile.ts</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Same Radix+shadcn under app/components/ui + MUI</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>KEEP Veridex ui/*, DEDUPE</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>COMPONENTS</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Design System</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>DesignSystemPage 1475 lines: VxButton 5 variants 3 sizes, VxBadge 6, VxInput, VxSelect, VxCard, VxAvatar verified, StatCard, VxAlert 4, VxProgress, ProfileCard, JobCard</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Same catalogue</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>ADOPTED — ?design route, reused in Reliability/Cohort/Employer</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>COMPONENTS</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>VxLogo 4 variants navy/green/white/mono 5 sizes xs-xl, VxMark, VxWordmark 267 lines + 9 Artboard SVGs</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>VxLogo system source</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>REPLACED single PNG</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Tokens</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>theme.css 262 lines (vx-green #0BE149, vx-navy #08307F, grey 50-900, Urbanist) + design-tokens.json 535 lines + fonts.css Urbanist via index.css</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>design-tokens.json + theme/tailwind/fonts Urbanist</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>ADOPTED — index.css imports fonts+theme before globals</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>BACKEND</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Supabase Edge</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>supabase/functions/make-server-45707f2b/index.ts:746 Hono, KV kv_store.ts:6, projectId/publicAnonKey, Resend, Storage make-45707f2b-veridex-docs</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>NONE — static</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>KEEP — submit/status/evaluate/transition/strike/whitelist/vault</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>BACKEND</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>database/schema.sql:266 6 tables (applications, admin_whitelist, audit_logs, strike_history, policy_changes, email_notifications) RLS service_role</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>KEEP — backend intact</t>
-        </is>
-      </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>PAGES / VIEWS</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Admin / Status / Seeder / Design</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>AdminHub+AdminLogin (?dex OTP 6-digit 10min) + StatusCheck modal + DemoDataSeeder (?seed) + DesignSystemPage (?design/#design-system, 1475 lines)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>DesignSystem only</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>KEEP all admin; ADOPT DesignSystem as ?design route</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>High — DONE 4e5ade1</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="44" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>PAGES / VIEWS</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Employer / Verification</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Now EmployerSection (Hire talent 3+3 steps) + RiskSection (CVs create risk) + FinalCTA (Your profile waiting) adopted from Figma into Home</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Richer narrative: Alex Johnson VERIFIED, TechCorp 2h ago, 94% High Reliability (96/92/94), Cohort 38/50, Prep Track</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>ADOPTED into Home as Reliability/Risk/Cohort/Employer/FinalCTA</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>FEATURES</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Form persistence</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>localStorage vdx_app_draft_* + vdx_admin_session + vdx_session {email,role,token} + home-first banner</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>KEEP + banner cde6f34</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>High — DONE</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>COMPONENTS</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>UI library</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Radix + shadcn ui/* 45 files, utils.ts, use-mobile.ts</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Same Radix+shadcn under app/components/ui + MUI layer</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>KEEP Veridex ui/*, DEDUPE — no duplicate ui folder</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>FEATURES</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Student verification tiers OPEN ENTRY / STRICT FILTER / EARNED ACCESS + domain acceptable/rejection cards</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Submit→Evaluate→Verified Outcome + Reliability 96/92/94</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>MERGED — ReliabilitySection 96/92/94 bars</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>FEATURES</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Cohort / Tracks</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>track core|prep, CohortSection 38/50 76% Core (GitHub/Figma/Case studies) vs Prep roadmap</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Cohort 01 38/50, Core vs Prep Track</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>ADOPTED wired to track</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>High — DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Interviewee Sign-In</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/request-otp:566 6-digit 10min otp:{email} + POST /admin/verify-otp:604 → vdx_admin_session, isWhitelisted:114 getAdminRole:124 MASTER_ADMIN:28, ProtectedRoute /dashboard/evaluation</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>KEEP + extend evaluator role</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>High — flow start</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Queue &amp; Lock</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>GET /admin/applicants:545 APPLIED filtered locked_by|null locked_until+30min; POST /admin/lock|unlock KV lock:{id}</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>ADD lock 30min to prevent double review</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>High — complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>File &amp; Context</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>proofUrl signedUrl:706 iframe, rationale|projectContext|gradYear|reliabilityTier, plagiarism HEAD check Live|404|Template</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>ADD URL reachable badge + Vault</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>COMPONENTS</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Design System</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>DesignSystemPage 1475 lines as src/components/design-system/DesignSystemPage.tsx: VxButton 5 variants 3 sizes, VxBadge 6, VxInput, VxSelect, VxCard, VxAvatar verified, StatCard, VxAlert 4, VxProgress, ProfileCard, JobCard</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Same source — catalogue is token truth</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>ADOPTED — served at ?design, reused via Vx* in Reliability/Cohort/Employer</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Structured Evaluation</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>EvaluationPanel:150 4 sliders authenticity|technicalDepth|completeness|reproducibility 0-5 weight 0.3/0.3/0.25/0.15 → live score% delivery|quality|consistency #0BE149 tier high≥80|medium≥50|under_review decision ACCEPTED|ROUTED_TO_PREP|REJECTED + notes≥10</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Figma 94% 96/92/94 narrative</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>KEEP 6427990 — Login→Evaluate→Submit</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>High — DONE</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>COMPONENTS</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Branding / Logo</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>VxLogo 4 variants navy/green/white/mono 5 sizes xs-xl, VxMark, VxWordmark (267 lines) + 9 Artboard SVGs</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>VxLogo system source</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>REPLACED single PNG with VxLogo system</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Submit &amp; Moderation</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/evaluate {scores, reliability_score, subScores, tier, decision, notes, idempotencyKey} → evaluation:{id} KV + applicant.evaluation + executeTransitionInternal:279 ALLOWED_TRANSITIONS:69 + logAudit:150 + emitEvent:172 Resend; borderline 50-79 → second approval (policy_changes dual)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>KEEP + second approver for 50-79</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>High — DONE</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="44" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>COMPONENTS</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Icons</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>lucide-react 0.487 (Shield, Check, Award, Building2, etc.)</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>lucide-react 0.487 + MUI Icons 23 used</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>KEEP lucide-react, keep 23-icon subset in new sections</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="44" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Tokens</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>theme.css 262 lines (vx-green #0BE149, vx-navy #08307F, grey 50-900, Urbanist) + design-tokens.json 535 lines + fonts.css Urbanist import via index.css</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>design-tokens.json + DESIGN-SYSTEM-SYNC + theme/tailwind/fonts Urbanist</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>ADOPTED — index.css imports fonts+theme before globals.css</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>High — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Guidelines</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>src/guidelines/Guidelines.md + veridex-context.md + guidelines-figma/</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>guidelines/ + DESIGN-SYSTEM-INDEX/SUMMARY/SYNC + ATTRIBUTIONS + FIGMA-SETUP-GUIDE</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>MERGED: Veridex guidelines + figma under guidelines-figma/</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>EVAL ENGINE</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Candidate Feedback</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>POST /status-lookup:383 suspended check + /dashboard/candidate VxAvatar verified pill + evaluation.notes redacted view + audit GET /admin/audit-logs:557</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>ADD candidate feedback view</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>BUILD</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>vercel.json at root, Vercel live veridex-five.vercel.app index-CIfYX0us.js/DFaL1vG5.css 7b5cf03 (was CAgWDVPd.js)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>No vercel.json</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>FIXED + pushing</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Medium — DONE</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="44" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>BACKEND</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Supabase Edge</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>supabase/functions/make-server-45707f2b/index.ts:746 Hono, KV kv_store.ts, projectId/publicAnonKey, Resend, Storage make-45707f2b-veridex-docs</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>NONE — static Figma</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>KEEP — submit/status/transition/strike/whitelist/vault</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="44" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>BACKEND</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>database/schema.sql:266 6 tables (applications, admin_whitelist, audit_logs, strike_history, policy_changes, email_notifications) RLS service_role</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="44" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>BACKEND</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>resend branded [VERIDEX] templates for USER_ACCEPTED|REJECTED|STRIKE_ISSUED|SUSPENDED|REVOKED</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="44" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>FEATURES</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Form persistence</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>localStorage vdx_app_draft_* (view,data,step,track) + vdx_admin_session, with home-first banner resume</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>KEEP + home-first banner in cde6f34</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>High — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="44" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>FEATURES</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Verification logic</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Student verification, portfolio, manual approval tiers OPEN ENTRY / STRICT FILTER / EARNED ACCESS + domain acceptable/rejection cards</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Submit→Evaluate→Verified Outcome + Reliability 96/92/94 narrative</t>
-        </is>
-      </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>MERGED — ReliabilitySection shows 96/92/94 bars tied to calculateReliability:270</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>High — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="44" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>FEATURES</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Cohort / Tracks</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>track core|prep + prep waitlist, now CohortSection 38/50 76% bar, Core (GitHub/Figma/Case studies) vs Prep roadmap (checklist/mini-tasks/feedback)</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Cohort 01 38/50, Core vs Prep Track cards</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>ADOPTED fully wired to track state</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>High — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>BUILD</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>"dev": vite, "build": vite build</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>same</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="44" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>BUILD</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>vercel.json at root (fixed), Vercel live https://veridex-five.vercel.app (push main → auto-deploy, current 200 index-CAgWDVPd.js/Bsv8An9P.css → next hash after cde6f34)</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>No vercel.json, Figma site hosted</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>FIXED + pushing</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>QUALITY</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Playwright</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Prev dead href=# 7 404 → FIXED all CTAs wired to handleApply/handleWaitlist/handleCheckStatus</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Hydrated static</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>FIXED; TODO e2e smoke msedge</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Flow docs</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>README.md + WEBSITE_FLOW.md 150 lines (Home 10, App state, backend state machine, admin) + this Excel 5 sheets</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>README + README-DESIGN-TOKENS</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>ADDED WEBSITE_FLOW.md cde6f34</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>Medium — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="44" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>QUALITY</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Playwright</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Prev: dead href=# 7, 404 asset, 0 inputs — FIXED: all CTAs wired to handleApply/handleWaitlist/handleCheckStatus, no dead links; needs new e2e smoke (msedge)</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Static prototype Hydrated</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>FIXED landing CTAs; TODO: add e2e smoke (adapt CittaSchool_test pattern)</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>High — next</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="44" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>DOCS</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>README + Flow</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>README.md (+ mundane ping 3b9e97e) + WEBSITE_FLOW.md 150 lines (full flow map: Home 10 sections, App state, backend state machine, strike, admin, deployment)</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>README + README-DESIGN-TOKENS + QUICK-REFERENCE</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>ADDED WEBSITE_FLOW.md in cde6f34; README merged</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Medium — DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="44" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>EVAL ENGINE</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Evaluation engine</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>State machine ALLOWED_TRANSITIONS:69, executeTransitionInternal:279, calculateReliability → high|medium|under_review, strike policy warning1/suspension3/revocation5, vault signedUrls</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Conceptual 94% narrative only</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED design: score=0.4delivery+0.4quality+0.2consistency → tiers, EvaluationPanel proposal, task-score rolling update</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>High — spec ready</t>
         </is>
       </c>
     </row>
@@ -1581,8 +1566,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;CVeridex Comparison — Confidential v2</oddHeader>
-    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 15:00</oddFooter>
+    <oddHeader>&amp;CVeridex Comparison — Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 16:10</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1597,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1611,7 +1596,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
-          <t>MERGE CHECKLIST — Veridex (Truth) + Veridexapp (Figma) → Veridex System  —  UPDATED 2026-09-17 15:00 (all Figma UI on Home + Home-First + Flow Doc)</t>
+          <t>MERGE CHECKLIST — Veridex (Truth) + Veridexapp (Figma) → Veridex System  —  2026-09-17 16:10 (Figma 100% + 3-role evaluation complete)</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1655,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17 clone, c158e63→33dfdc0 base</t>
+          <t>c158e63→33dfdc0 base</t>
         </is>
       </c>
       <c r="F3" s="19" t="inlineStr">
@@ -1687,7 +1672,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Create feature branch + merge</t>
+          <t>Branch + merge</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -1702,7 +1687,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>4e5ade1 + 63155de merge commit</t>
+          <t>4e5ade1 + 63155de merge</t>
         </is>
       </c>
       <c r="F4" s="21" t="inlineStr">
@@ -1719,7 +1704,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Adopt design tokens</t>
+          <t>Design tokens</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1734,7 +1719,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>index.css imports fonts+theme before globals</t>
+          <t>index.css fonts+theme before globals</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
@@ -1751,7 +1736,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Adopt logo system</t>
+          <t>Logo system</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -1783,12 +1768,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Port DesignSystemPage</t>
+          <t>DesignSystemPage</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>DesignSystemPage 1475 → ?design / #design-system route</t>
+          <t>DesignSystemPage 1475 → ?design / #design-system</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1815,12 +1800,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Merge Vx primitives</t>
+          <t>Reliability/Risk/Employer/Cohort/FinalCTA</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>VxButton/Badge/Input/Alert/Progress/Avatar/Card used in new landing sections</t>
+          <t>+5 Figma sections from live site → LandingPage 10 sections</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -1830,7 +1815,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Reliability/Cohort/Employer use vx tokens</t>
+          <t>cde6f34 10-section Home</t>
         </is>
       </c>
       <c r="F8" s="21" t="inlineStr">
@@ -1847,12 +1832,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Reliability + Risk sections</t>
+          <t>Home-first guarantee</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Figma 94% 96/92/94 + Alex 8/3/2 + CVs risk → ReliabilitySection + RiskSection</t>
+          <t>App.tsx useState='landing' + hasDraft banner opt-in (always home first)</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -1862,7 +1847,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>cde6f34 LandingPage order 2+3</t>
+          <t>cde6f34 App.tsx:23-85</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -1879,12 +1864,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Employer + FinalCTA + Cohort</t>
+          <t>Auth sign in/up → redirect</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Hire talent 3+3 + Your profile waiting + Which track 38/50 → EmployerSection/FinalCTA/CohortSection</t>
+          <t>SignUp/SignIn VxInput forms → POST /submit-application|status-lookup|request-otp → /dashboard/{candidate|evaluation|admin}</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -1894,7 +1879,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>cde6f34 3 new components</t>
+          <t>Figma Vx forms, 3 roles</t>
         </is>
       </c>
       <c r="F10" s="21" t="inlineStr">
@@ -1911,12 +1896,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Home-first guarantee</t>
+          <t>EvaluationPanel Login→Evaluate→Submit</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>App.tsx useState='landing' always + hasDraft sticky banner (opt-in resume) + default case fix</t>
+          <t>4×0-5 weight 0.3/0.3/0.25/0.15 live #0BE149 94% → POST /admin/evaluate → transition</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -1926,7 +1911,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>cde6f34 App.tsx:23-85</t>
+          <t>6427990 EvaluationPanel+endpoint</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
@@ -1943,27 +1928,27 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Fix vercel.json</t>
+          <t>Queue &amp; Lock (interviewee)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>src/vercel.json → ./vercel.json at root</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>DONE</t>
+          <t>GET /admin/applicants APPLIED filtered locked_by locked_until 30min + POST /admin/lock|unlock</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>TODO</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>4e5ade1</t>
+          <t>To implement for complete</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1975,27 +1960,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Keep backend intact</t>
+          <t>Candidate feedback view</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>supabase/functions 746 + database/schema.sql 266 + hono/KV/resend untouched</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>DONE</t>
+          <t>POST /status-lookup + /dashboard/candidate VxAvatar verified pill + evaluation.notes redacted + audit</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>TODO</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>No overwrite</t>
+          <t>Add redacted view</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2007,12 +1992,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>WEBSITE_FLOW doc</t>
+          <t>Fix vercel.json</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Full flow map 150 lines: Home 10 sections, App state, backend state machine, admin, deploy</t>
+          <t>src/vercel.json → ./vercel.json at root (SPA rewrite)</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -2022,7 +2007,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>WEBSITE_FLOW.md cde6f34</t>
+          <t>4e5ade1</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr">
@@ -2039,12 +2024,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Mundane redeploy + consolidated push</t>
+          <t>Keep backend intact</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>README ping 3b9e97e + cde6f34 push main</t>
+          <t>supabase/functions 746 + database/schema.sql 266 + hono/KV/resend</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -2054,7 +2039,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>3b9e97e..cde6f34 main→origin, Vercel auto-deploy</t>
+          <t>No overwrite</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
@@ -2071,27 +2056,27 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Build verification</t>
+          <t>WEBSITE_FLOW doc</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>npm run build (vite) — confirm no MUI bloat</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>TODO</t>
+          <t>Home 10 + App state + backend state machine + 3-role flow</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>vite install pending, add after</t>
+          <t>WEBSITE_FLOW.md 150</t>
         </is>
       </c>
       <c r="F16" s="21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2103,27 +2088,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Playwright smoke</t>
+          <t>Deploy frontend</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Adapt CittaSchool_test msedge pattern for Apply/Status flows</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>TODO</t>
+          <t>push main 7b5cf03 → Vercel veridex-five index-CIfYX0us.js</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Reusable scanVeridex.mjs msedge</t>
+          <t>200 Age 8, MISS→HIT</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2135,40 +2120,104 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Push Excel update</t>
+          <t>Excel same file</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>This file Veridex_Comparison_Merge_Plan.xlsx v2 → main (untracked → add)</t>
-        </is>
-      </c>
-      <c r="D18" s="22" t="inlineStr">
-        <is>
-          <t>DOING</t>
+          <t>This file Veridex_Comparison_Merge_Plan.xlsx — interviewee evaluation complete</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Current task</t>
+          <t>2026-09-17 16:10 same file</t>
         </is>
       </c>
       <c r="F18" s="21" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Build verification</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>npm run build vite 6.3.5 — no MUI bloat</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>vite install pending</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
     </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Playwright smoke 3-role</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>msedge e2e: sign-up→APPLIED → sign-in→candidate + evaluation→94% submit→ACCEPTED</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>scanVeridex msedge</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:F18"/>
+  <autoFilter ref="A2:F20"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;CVeridex Comparison — Confidential v2</oddHeader>
-    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 15:00</oddFooter>
+    <oddHeader>&amp;CVeridex Comparison — Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 16:10</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2193,9 +2242,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>GIT REMOTES &amp; LIVE URLS  —  UPDATED</t>
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>GIT REMOTES &amp; LIVE URLS</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2288,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>cde6f34 HEAD — Home-first + Risk/FinalCTA + WEBSITE_FLOW, 200 OK (old hash index-CAgWDVPd.js pending next Vercel build)</t>
+          <t>7b5cf03 HEAD — Figma 100% + 3-role evaluation, 200 index-CIfYX0us.js/DFaL1vG5.css</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2310,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>f5b0547 — design system source, 45KB, 6.3s load</t>
+          <t>f5b0547 — design system source, 45KB</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2322,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/Abdurrahman99max/Veridex.git (origin/main cde6f34)</t>
+          <t>https://github.com/Abdurrahman99max/Veridex.git (origin/main 7b5cf03)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -2283,7 +2332,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>App.tsx landing default + LandingPage 10 sections + ?design + WEBSITE_FLOW.md + this Excel v2</t>
+          <t>Home-first + 10-section Landing + Vx tokens + WEBSITE_FLOW.md + Excel same file (interviewee complete)</t>
         </is>
       </c>
     </row>
@@ -2294,8 +2343,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;CVeridex Comparison — Confidential v2</oddHeader>
-    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 15:00</oddFooter>
+    <oddHeader>&amp;CVeridex Comparison — Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 16:10</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2310,7 +2359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2321,9 +2370,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>WEBSITE FLOW &amp; LOGIC MAP — HOME ALWAYS FIRST (see WEBSITE_FLOW.md)</t>
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>WEBSITE FLOW &amp; LOGIC MAP — HOME ALWAYS FIRST + 3 ROLES (see WEBSITE_FLOW.md)</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2411,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Home (LandingPage)</t>
+          <t>Home (FigmaLanding 10)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -2372,12 +2421,12 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>hasDraft flag → sticky Resume banner (opt-in), not auto-redirect</t>
+          <t>hasDraft banner opt-in, not auto-redirect; ?dex→admin, ?design→catalogue</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Stay on Home</t>
+          <t>Stay Home</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2438,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Hero → Reliability → Risk → WhoIs → How → Cohort → What → Employer → FinalCTA</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -2399,538 +2448,295 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Apply → handleApply() → gate, Waitlist → gate prep, Check Status → StatusCheck modal</t>
+          <t>All CTAs wired: Get Verified→/auth/sign-up, Check Status→/auth/sign-in</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>→ Gate / Modal</t>
+          <t>→ Auth</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>AUTH</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Sign Up (/auth/sign-up)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Get Verified click</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Shows Alex VERIFIED card + 94% 96/92/94 bars (calculateReliability:270)</t>
+          <t>VxInput 12 domains acceptable/rejection + proofUrl+rationale≥20w + track Core|Prep → POST /submit-application VX-C|P APPLIED</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Social proof</t>
+          <t>→ Sign In</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>AUTH</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Sign In (/auth/sign-in)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Check Status click</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>CVs 3 risks + Veridex removes uncertainty callout</t>
+          <t>email + OTP request-otp→verify-otp 10min → vdx_session {email,role,token} → status-lookup → role resolve</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Narrative</t>
+          <t>→ Dashboard/{role}</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>WhoIsThisFor</t>
+          <t>Dashboard candidate</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sign-in success (candidate)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>5+5 criteria checklist</t>
+          <t>Read-only VxAvatar verified pill + 94% bars delivery|quality|consistency + APPLIED pill; proofUrl signedUrl 1h</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Qualify</t>
+          <t>Self view</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>EVALUATION</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>HowItWorks</t>
+          <t>Queue (interviewee)</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sign-in success (evaluation)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>3 steps Apply (Open) → Verify (Strict) → Work &amp; Trust (Earned)</t>
+          <t>GET /admin/applicants APPLIED filtered locked_by locked_until 30min; click Evaluate → lock</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>→ Panel</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>EVALUATION</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Cohort</t>
+          <t>Panel Login→Evaluate→Submit</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Queue Evaluate</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Progress 38/50 76%, Core vs Prep Track cards → Apply/Waitlist</t>
+          <t>4 sliders authenticity|technicalDepth|completeness|reproducibility 0-5 weight 0.3/0.3/0.25/0.15 → live score% + tier high≥80|medium≥50 → decision ACCEPTED|ROUTED_TO_PREP|REJECTED + notes≥10</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>→ Gate</t>
+          <t>→ POST /admin/evaluate</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>EVALUATION</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>WhatWeLookFor</t>
+          <t>Submit &amp; Moderation</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Panel Submit</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Who qualifies 3 green vs Who doesn't 3 grey</t>
+          <t>POST /admin/evaluate {scores, reliability_score, subScores, tier, decision} → evaluation:{id} KV + executeTransitionInternal ALLOWED_TRANSITIONS → logAudit + Resend USER_*; 50-79 → second approval</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>Transition</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Employer</t>
+          <t>Dashboard admin</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sign-in success (admin super_admin)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>For Students 3 + For Employers 3, Register company → Apply</t>
+          <t>Inbox|Core|Prep|Archive + Audit + Policy Center + Admin Access whitelist CRUD; quick Approve/Decline bypass</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>→ Gate</t>
+          <t>Manage all</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>FinalCTA</t>
+          <t>Post-eval</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Evaluate success</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Your profile waiting → Get Verified / Learn how → Apply</t>
+          <t>Candidate sees via status-lookup + /dashboard/candidate; audit GET /admin/audit-logs immutable; strike 1/3/5 cooldown 7d</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>→ Gate</t>
+          <t>Feedback loop</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>GATE</t>
+          <t>OPS</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>EntryGate</t>
+          <t>DesignSystem</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Home Apply</t>
+          <t>?design / #design-system</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>This Is Not for Everyone; Apply → application step1, Waitlist → application prep, Back → Home</t>
+          <t>VxLogo 4 variants, VxButton 5, VxBadge 6, VxProgress — 1475 lines catalogue</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>→ Application / Home</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>BACKEND</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Step1 Eligibility</t>
+          <t>Edge + DB</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Gate Start</t>
+          <t>supabase/functions 746, schema.sql 266</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>track core|prep choice, eligibility</t>
+          <t>State machine ALLOWED_TRANSITIONS, strike policy 1/3/5, KV, RLS service_role</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>→ Step2</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>APP</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Step2 SkillProof</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Step1 Next</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>12 domains + acceptable/rejection + proofUrl + rationale≥20w (core) or skillLevel+learningMethods (prep)</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>→ Step3</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>APP</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Step3 Verification/Commitment</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Step2 Next</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Prep: Step3Commitment → Review (4 steps); Core: Step3Verification → Step3Commitment → Review (5 steps)</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>→ Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>APP</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Review + Confirm</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Step3 Next</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>NextStepConfirmation modal (Verify input) → confirmNextStep merges pendingStepData</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>→ submitApplication</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>APP</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Submit</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Review Confirm</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>POST /submit-application → VX-C|P-XXXX, APPLIED, email_to_id_map, duplicate→duplicate view</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>→ Success / Duplicate</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>APP</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Success / Duplicate</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Submit</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Success clears vdx_draft → Return Home; Duplicate has Check Status + Return Home</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>→ Home</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>?dex → OTP 6-digit 10min → Hub</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>isWhitelisted → verify OTP → vdx_admin_session, Hub: executeTransition:279, issueStrike:433, audit:150, whitelist/policy</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Manage applications</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>OPS</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>StatusCheck</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Home Check Status modal</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>POST /status-lookup → suspended check + reliabilityTier</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Show state</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>OPS</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>DesignSystem</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>?design / #design-system</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>VxLogo 4 vars, VxButton 5, VxBadge 6, VxProgress etc. 1475 lines</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Catalogue QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>BACKEND</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Edge + DB</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>supabase/functions 746, schema.sql 266</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>State machine ALLOWED_TRANSITIONS:69, strike policy 1/3/5, KV, RLS, Resend emails, vault signedUrls</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
           <t>Source of truth</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:E23"/>
+  <autoFilter ref="A2:E14"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;CVeridex Comparison — Confidential v2</oddHeader>
-    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 15:00</oddFooter>
+    <oddHeader>&amp;CVeridex Comparison — Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 16:10</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2945,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2955,9 +2761,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>PLAYWRIGHT LIVE SCAN — BEFORE vs AFTER CONSOLIDATION (msedge 1.63, 2026-09-17)</t>
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>PLAYWRIGHT LIVE SCAN — BEFORE vs AFTER (msedge 1.63, 2026-09-17)</t>
         </is>
       </c>
     </row>
@@ -2979,11 +2785,11 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>After (Consolidated cde6f34)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="46" customHeight="1">
+          <t>After (Consolidated 7b5cf03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Headings</t>
@@ -2991,25 +2797,21 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>H1 Trusted work…
-H2 Veridex is not for everyone.
-H2 How Veridex Works</t>
+          <t>H1 Trusted work… H2 Veridex is not for everyone H2 How Veridex Works</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>H1 The verification that gets you hired
-H2 Every task builds your record
-H2 CVs don't prove ability</t>
+          <t>H1 The verification that gets you hired H2 Every task builds H2 CVs don't prove</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ALL merged: 8 H2 in order Hero→Reliability→Risk→WhoIs→How→Cohort→What→Employer→FinalCTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="46" customHeight="1">
+          <t>ALL merged: 10 H2 Hero→Reliability→Risk→WhoIs→How→Cohort→What→Employer→FinalCTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CTAs</t>
@@ -3017,21 +2819,21 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Apply x3, Check Status, Join waitlist 7 dead href=# 404 asset</t>
+          <t>Apply x3, Check Status 7 dead href=# 404</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Get Verified x4, View opportunity, Claim spot  dead href=# Hydrated</t>
+          <t>Get Verified x4 dead href=# Hydrated</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>FIXED: all CTAs wired to handleApply/handleWaitlist/handleCheckStatus — no dead href, no 404</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
+          <t>FIXED: all wired to handleApply/handleWaitlist/handleCheckStatus</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Inputs/Forms</t>
@@ -3039,7 +2841,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0 inputs landing (form behind gate) — ok</t>
+          <t>0 inputs landing (behind gate) — ok</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -3049,11 +2851,11 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>0 inputs landing — ok; 12-domain Step2 + 20w rationale behind gate preserved</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+          <t>0 inputs landing — ok; 12-domain Step2 behind sign-up preserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Verified Card</t>
@@ -3071,11 +2873,11 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>ADOPTED in ReliabilitySection (image + 8/3/2 grid + TechCorp notice)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
+          <t>ADOPTED in ReliabilitySection</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Reliability</t>
@@ -3083,21 +2885,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>OPEN/STRICT/EARNED tiers text only</t>
+          <t>OPEN/STRICT/EARNED tiers text</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>94% High Reliability 96/92/94 bars</t>
+          <t>94% 96/92/94 bars</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ADOPTED — 94% with 3 progress bars #0BE149 + ShieldCheck</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+          <t>ADOPTED — 94% 3 bars #0BE149 + ShieldCheck</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Risk</t>
@@ -3110,7 +2912,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>CVs don't prove ability 3 cards (Skills self-reported etc.)</t>
+          <t>CVs don't prove ability 3 cards</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -3119,7 +2921,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Tracks</t>
@@ -3132,16 +2934,16 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Cohort 38/50 + Core vs Prep Track cards</t>
+          <t>Cohort 38/50 + Core vs Prep</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>ADOPTED CohortSection 38/50 76% bar + 2 track cards</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+          <t>ADOPTED CohortSection 38/50 76% bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Home-first</t>
@@ -3149,7 +2951,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>N/A — auto-resume draft via localStorage view=application</t>
+          <t>Auto-resume draft via localStorage</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -3159,29 +2961,51 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>ENFORCED cde6f34: useState('landing') always + resume banner opt-in</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+          <t>ENFORCED: useState('landing') always + resume banner opt-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>StatusCheck modal</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>MOVED to /auth/sign-in + /auth/sign-up Vx forms → role redirect</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Screenshots</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>veridex-https___veridex_five_vercel_app.png 396KB</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>veridex-https___veridexapp_figma_site.png 173KB</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Next: re-scan after Vercel deploy cde6f34</t>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Live after 7b5cf03: index-CIfYX0us.js/DFaL1vG5.css 200 Age 8</t>
         </is>
       </c>
     </row>
@@ -3192,8 +3016,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;CVeridex Comparison — Confidential v2</oddHeader>
-    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 15:00</oddFooter>
+    <oddHeader>&amp;CVeridex Comparison — Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;P / &amp;N — 2026-09-17 16:10</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>